<commit_message>
Actualización rutas y snomed
</commit_message>
<xml_diff>
--- a/Rutas Carpetas/catalogo_rutas.xlsx
+++ b/Rutas Carpetas/catalogo_rutas.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\francisca.tapia\Desktop\Repositorios GITHUB\HTML_ISP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\francisca.tapia\Desktop\Repositorios GITHUB\HTML_ISP\Rutas Carpetas\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12312"/>
   </bookViews>
   <sheets>
-    <sheet name="query (1)" sheetId="1" r:id="rId1"/>
+    <sheet name="query" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="query__1" localSheetId="0" hidden="1">'query (1)'!$A$1:$C$74</definedName>
+    <definedName name="query" localSheetId="0" hidden="1">query!$A$1:$C$58</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -23,14 +23,14 @@
 
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
 <connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <connection id="1" odcFile="C:\Users\francisca.tapia\Downloads\query (1).iqy" keepAlive="1" name="query (1)" type="5" refreshedVersion="6" minRefreshableVersion="3" saveData="1">
+  <connection id="1" odcFile="C:\Users\francisca.tapia\Downloads\query.iqy" keepAlive="1" name="query" type="5" refreshedVersion="6" minRefreshableVersion="3" saveData="1">
     <dbPr connection="Provider=Microsoft.Office.List.OLEDB.2.0;Data Source=&quot;&quot;;ApplicationName=Excel;Version=12.0.0.0" command="&lt;LIST&gt;&lt;VIEWGUID&gt;23F50D66-6C9D-4A71-8778-D9E910B98ABB&lt;/VIEWGUID&gt;&lt;LISTNAME&gt;0328af18-8582-4575-9620-6f27dc8d3768&lt;/LISTNAME&gt;&lt;LISTWEB&gt;https://ispchcl.sharepoint.com/sites/VigilanciaEpidemiolgicaSanitaria/_vti_bin&lt;/LISTWEB&gt;&lt;LISTSUBWEB&gt;&lt;/LISTSUBWEB&gt;&lt;ROOTFOLDER&gt;&lt;/ROOTFOLDER&gt;&lt;/LIST&gt;" commandType="5"/>
   </connection>
 </connections>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="174">
   <si>
     <t>SNOMED_CT</t>
   </si>
@@ -44,7 +44,7 @@
     <t>14590003</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/01-BICE-Bacterias Intracelulares y Cultivos Especiales/14590003-C. psittaci/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/14590003-C. psittaci/Datos Vigilancia</t>
   </si>
   <si>
     <t>Chlamydia trachomatis</t>
@@ -53,7 +53,7 @@
     <t>63938009</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/01-BICE-Bacterias Intracelulares y Cultivos Especiales/63938009-C. trachomatis/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/63938009-C. trachomatis/Datos Vigilancia</t>
   </si>
   <si>
     <t>Coxiella burnetii</t>
@@ -62,7 +62,7 @@
     <t>22533000</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/01-BICE-Bacterias Intracelulares y Cultivos Especiales/22533000-C. burnetii/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/22533000-C. burnetii/Datos Vigilancia</t>
   </si>
   <si>
     <t>Rickettsia spp</t>
@@ -71,7 +71,7 @@
     <t>62065006</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/01-BICE-Bacterias Intracelulares y Cultivos Especiales/62065006-Rickettsia spp/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/62065006-Rickettsia spp/Datos Vigilancia</t>
   </si>
   <si>
     <t>Brucella spp</t>
@@ -80,7 +80,7 @@
     <t>26250004</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/02-EMZ-Emergentes y zoonóticos/26250004-Brucella spp/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/26250004-Brucella spp/Datos Vigilancia</t>
   </si>
   <si>
     <t>Campylobacter spp</t>
@@ -89,7 +89,7 @@
     <t>35408001</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/02-EMZ-Emergentes y zoonóticos/35408001-Campylobacter spp/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/35408001-Campylobacter spp/Datos Vigilancia</t>
   </si>
   <si>
     <t>Leptospira</t>
@@ -98,7 +98,7 @@
     <t>26764003</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/02-EMZ-Emergentes y zoonóticos/26764003-Leptospira/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/26764003-Leptospira/Datos Vigilancia</t>
   </si>
   <si>
     <t>Escherichia coli enterohemorrágica (ECEH)</t>
@@ -107,7 +107,7 @@
     <t>838549008</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/03-ETA-Enfermedades Transmitidas por Alimentos/838549008-E. coli/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/838549008-E. coli/Datos Vigilancia</t>
   </si>
   <si>
     <t>Salmonella spp</t>
@@ -116,7 +116,7 @@
     <t>27268008</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/03-ETA-Enfermedades Transmitidas por Alimentos/27268008-Salmonella spp/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/27268008-Salmonella spp/Datos Vigilancia</t>
   </si>
   <si>
     <t>Shigella spp</t>
@@ -125,7 +125,7 @@
     <t>77352002</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/03-ETA-Enfermedades Transmitidas por Alimentos/77352002-Shigella spp/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/77352002-Shigella spp/Datos Vigilancia</t>
   </si>
   <si>
     <t>Vibrio cholerae</t>
@@ -134,7 +134,7 @@
     <t>75953000</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/03-ETA-Enfermedades Transmitidas por Alimentos/75953000-V. cholerae/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/75953000-V. cholerae/Datos Vigilancia</t>
   </si>
   <si>
     <t>Vibrio parahaemolyticus</t>
@@ -143,7 +143,7 @@
     <t>11736008</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/03-ETA-Enfermedades Transmitidas por Alimentos/11736008-V. parahaemolyticus/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/11736008-V. parahaemolyticus/Datos Vigilancia</t>
   </si>
   <si>
     <t>Yersinia spp</t>
@@ -152,7 +152,7 @@
     <t>4668009</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/03-ETA-Enfermedades Transmitidas por Alimentos/4668009-Yersinia spp/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/4668009-Yersinia spp/Datos Vigilancia</t>
   </si>
   <si>
     <t>Neisseria gonorrhoeae</t>
@@ -161,7 +161,7 @@
     <t>68704007</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/05-ITS-Infecciones de Transmisión Sexual/68704007-N. gonorrhoeae/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/68704007-N. gonorrhoeae/Datos Vigilancia</t>
   </si>
   <si>
     <t>Neisseria meningitidis</t>
@@ -170,7 +170,7 @@
     <t>17872004</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/06-MEN-Meningitis Bacterianas/17872004-N. meningitidis/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/17872004-N. meningitidis/Datos Vigilancia</t>
   </si>
   <si>
     <t>Listeria monocytogenes</t>
@@ -179,7 +179,7 @@
     <t>36094007</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/06-MEN-Meningitis Bacterianas/36094007-L. monocytogenes/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/36094007-L. monocytogenes/Datos Vigilancia</t>
   </si>
   <si>
     <t>Streptococcus agalactiae</t>
@@ -188,7 +188,7 @@
     <t>43492007</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/06-MEN-Meningitis Bacterianas/43492007-S. Agalactiae/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/43492007-S. agalactiae/Datos Vigilancia</t>
   </si>
   <si>
     <t>Haemophilus influenzae</t>
@@ -197,7 +197,7 @@
     <t>44470000</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/06-MEN-Meningitis Bacterianas/44470000-H. influenzae/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/44470000-H. influenzae/Datos Vigilancia</t>
   </si>
   <si>
     <t>Streptococcus pyogenes</t>
@@ -206,7 +206,7 @@
     <t>80166006</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/06-MEN-Meningitis Bacterianas/80166006-S. pyogenes/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/80166006-S. pyogenes/Datos Vigilancia</t>
   </si>
   <si>
     <t>Streptococcus pneumoniae</t>
@@ -215,446 +215,340 @@
     <t>9861002</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/06-MEN-Meningitis Bacterianas/9861002-S. pneumoniae/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Bordetella Pertussis</t>
-  </si>
-  <si>
-    <t>5247005</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/08-MM-Microbiología Molecular/5247005-B. pertussis/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Legionella spp</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/9861002-S. pneumoniae/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>PCR Bordetella Pertussis</t>
+  </si>
+  <si>
+    <t>5247005_PCR</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/5247005-B. pertussis/Datos Vigilancia/PCR</t>
+  </si>
+  <si>
+    <t>PCR Legionella spp</t>
+  </si>
+  <si>
+    <t>7527002_PCR</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/7527002-Legionella spp/Datos Vigilancia/PCR</t>
+  </si>
+  <si>
+    <t>Hantavirus</t>
+  </si>
+  <si>
+    <t>442001008</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/442001008-Hanta/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>PCR Coxiella burnetii</t>
+  </si>
+  <si>
+    <t>22533000_PCR</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/22533000-C. burnetii/Datos Vigilancia/PCR</t>
+  </si>
+  <si>
+    <t>PCR Rickettsia spp</t>
+  </si>
+  <si>
+    <t>62065006_PCR</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/62065006-Rickettsia spp/Datos Vigilancia/PCR</t>
+  </si>
+  <si>
+    <t>PCR meningitis bacteriana cultivos negativos</t>
+  </si>
+  <si>
+    <t>7180009_PCR</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/0-Otros/PCR-Meningitis</t>
+  </si>
+  <si>
+    <t>Virus Dengue</t>
+  </si>
+  <si>
+    <t>34348001</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/34348001-Dengue/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Virus Hepatitis A</t>
+  </si>
+  <si>
+    <t>32452004</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/32452004-Hepatitis_A/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Virus Hepatitis B</t>
+  </si>
+  <si>
+    <t>81665004</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/81665004-Hepatitis_B/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Virus Hepatitis C</t>
+  </si>
+  <si>
+    <t>62944002</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/62944002-Hepatitis_C/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Virus HTLV I/II</t>
+  </si>
+  <si>
+    <t>77457007</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/77457007-HTLV/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Virus Papiloma Humano (VPH)</t>
+  </si>
+  <si>
+    <t>9482002</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/9482002-Papiloma_Humano(VPH)/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Virus Parotiditis</t>
+  </si>
+  <si>
+    <t>50384007</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/50384007-Parotiditis/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Virus Rabia</t>
+  </si>
+  <si>
+    <t>59881000</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/59881000-Rabia/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Creutzfeldt-Jakob</t>
+  </si>
+  <si>
+    <t>88520007</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/88520007-Creutzfeldt-Jakob/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Influenza y otros virus respiratorios</t>
+  </si>
+  <si>
+    <t>725894000</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/725894000-Influenza_y_otros_virus_respiratorios/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Norovirus</t>
+  </si>
+  <si>
+    <t>407359000</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/407359000-Norovirus/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Poliovirus (PFA)</t>
+  </si>
+  <si>
+    <t>44172002</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/44172002-Poliovirus/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Rotavirus</t>
+  </si>
+  <si>
+    <t>417542000</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/417542000-Rotavirus/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Rubeola congénita (SRC)</t>
+  </si>
+  <si>
+    <t>8059002</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/8059002-Rubeola Congénita/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Plasmodium spp (Malaria)</t>
+  </si>
+  <si>
+    <t>34706006</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/02-Parasitos/34706006-Plasmodium_spp(Malaria)/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Trichinella spiralis (Triquinosis)</t>
+  </si>
+  <si>
+    <t>16439004</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/02-Parasitos/16439004-Trichinella_spiralis(Triquinosis)/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Trypanosoma cruzi (Chagas)</t>
+  </si>
+  <si>
+    <t>88274000</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/02-Parasitos/88274000-Trypanosoma_cruzi(Chagas)/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Candida spp.</t>
+  </si>
+  <si>
+    <t>3265006</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/04-Hongos/3265006-Candida_spp/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Bacillus spp.</t>
+  </si>
+  <si>
+    <t>44762009</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/44762009-Bacillus/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Clostridium botulinico</t>
+  </si>
+  <si>
+    <t>13080008</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/13080008-C.botulinico/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Mycobacterium leprae</t>
+  </si>
+  <si>
+    <t>58242002</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/58242002-M.leprae/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Clostridium tetanicum</t>
+  </si>
+  <si>
+    <t>30917009</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/30917009-C.tetanicum/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Corynebacterium Diphtheriae</t>
+  </si>
+  <si>
+    <t>5851001</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/5851001-C.Diphtheriae/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Mycobacterium tuberculosis</t>
+  </si>
+  <si>
+    <t>113861009</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/113861009-M.tuberculosis/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>VIH</t>
+  </si>
+  <si>
+    <t>19030005</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/19030005-VIH/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Salmonella typhi</t>
+  </si>
+  <si>
+    <t>5595000</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/5595000_SalmonellaT/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Cisticercosis</t>
+  </si>
+  <si>
+    <t>17966003</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/02-Parasitos/17966003-Cisticercosis/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Hidatidosis</t>
+  </si>
+  <si>
+    <t>243672005</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/02-Parasitos/243672005-Hidatidosis/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Leishmaniasis</t>
   </si>
   <si>
     <t>7527002</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/08-MM-Microbiología Molecular/7527002-Legionella spp/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Hantavirus</t>
-  </si>
-  <si>
-    <t>442001008</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/02-Virus Hepaticos y Emergentes/442001008-Hanta/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>PCR Bordetella Pertussis</t>
-  </si>
-  <si>
-    <t>5247005_PCR</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/08-MM-Microbiología Molecular/5247005-B. pertussis/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t>PCR Coxiella burnetii</t>
-  </si>
-  <si>
-    <t>22533000_PCR</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/01-BICE-Bacterias Intracelulares y Cultivos Especiales/22533000-C. burnetii/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t>PCR Legionella spp</t>
-  </si>
-  <si>
-    <t>7527002_PCR</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/08-MM-Microbiología Molecular/7527002-Legionella spp/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t>PCR Rickettsia spp</t>
+    <t>/Documentos compartidos/Biomedico/02-Parasitos/7527002-Leishmaniasis/Datos Vigilancia</t>
+  </si>
+  <si>
+    <t>Diarrea</t>
   </si>
   <si>
     <t>PENDIENTE</t>
   </si>
   <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/01-BICE-Bacterias Intracelulares y Cultivos Especiales/62065006-Rickettsia spp/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t>PCR meningitis bacteriana cultivos negativos</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/06-MEN-Meningitis Bacterianas/PCR-MeningitisBacteriana</t>
-  </si>
-  <si>
-    <t>Virus Chikungunya</t>
-  </si>
-  <si>
-    <t>2423009</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/02-Virus Hepaticos y Emergentes/2423009-Chikungunya/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus del Nilo</t>
-  </si>
-  <si>
-    <t>57311007</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/02-Virus Hepaticos y Emergentes/57311007-Virus_del_Nilo/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus Dengue</t>
-  </si>
-  <si>
-    <t>34348001</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/02-Virus Hepaticos y Emergentes/34348001-Dengue/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus Fiebre Amarilla</t>
-  </si>
-  <si>
-    <t>26630006</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/02-Virus Hepaticos y Emergentes/26630006-Fiebre_Amarilla/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus Hepatitis A</t>
-  </si>
-  <si>
-    <t>32452004</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/02-Virus Hepaticos y Emergentes/32452004-Hepatitis_A/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus Hepatitis B</t>
-  </si>
-  <si>
-    <t>81665004</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/02-Virus Hepaticos y Emergentes/81665004-Hepatitis_B/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus Hepatitis C</t>
-  </si>
-  <si>
-    <t>62944002</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/02-Virus Hepaticos y Emergentes/62944002-Hepatitis_C/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus Hepatitis E</t>
-  </si>
-  <si>
-    <t>78475006</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/02-Virus Hepaticos y Emergentes/78475006-Hepatitis_E/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus HTLV I/II</t>
-  </si>
-  <si>
-    <t>77457007</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/03-Virus Oncogénicos/77457007-HTLV/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus Papiloma Humano</t>
-  </si>
-  <si>
-    <t>9482002</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/03-Virus Oncogénicos/9482002-Papiloma_Humano/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus Parotiditis</t>
-  </si>
-  <si>
-    <t>50384007</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/03-Virus Oncogénicos/50384007-Parotiditis/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus Rabia</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/04-Virus Rábico/PENDIENTE-Rabia/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus Varicela-Zoster</t>
-  </si>
-  <si>
-    <t>19551004</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/05-Virus Respiratorios y Exantemáticos/19551004-Varicela-Zoster/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Virus Zika</t>
-  </si>
-  <si>
-    <t>50471002</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/02-Virus Hepaticos y Emergentes/50471002-Zika/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Creutzfeldt-Jakob</t>
-  </si>
-  <si>
-    <t>88520007</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/03-Virus Oncogénicos/88520007-Creutzfeldt-Jakob/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Influenza y otros virus respiratorios</t>
-  </si>
-  <si>
-    <t>725894000</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/05-Virus Respiratorios y Exantemáticos/725894000-Influenza_y_otros_virus_respiratorios/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Norovirus</t>
-  </si>
-  <si>
-    <t>407359000</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/01-Virus Entéricos/407359000-Norovirus/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Poliovirus</t>
-  </si>
-  <si>
-    <t>44172002</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/01-Virus Entéricos/44172002-Poliovirus/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Rotavirus</t>
-  </si>
-  <si>
-    <t>417542000</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/01-Virus Entéricos/417542000-Rotavirus/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Rubivirus</t>
-  </si>
-  <si>
-    <t>45156000</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/05-Virus Respiratorios y Exantemáticos/45156000-Rubivirus/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Morbillivirus</t>
-  </si>
-  <si>
-    <t>83313003</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/05-Virus Respiratorios y Exantemáticos/83313003-Morbillivirus/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Plasmodium spp (Malaria)</t>
-  </si>
-  <si>
-    <t>34706006</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/02-Parasitos/34706006-Plasmodium_spp(Malaria)/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Trichinella spiralis (Triquinosis)</t>
-  </si>
-  <si>
-    <t>16439004</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/02-Parasitos/16439004-Trichinella_spiralis(Triquinosis)/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Trypanosoma cruzi (Chagas)</t>
-  </si>
-  <si>
-    <t>88274000</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/02-Parasitos/88274000-Trypanosoma_cruzi(Chagas)/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Candida spp.</t>
-  </si>
-  <si>
-    <t>3265006</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/04-Hongos/3265006-Candida_spp/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Bacillus spp.</t>
-  </si>
-  <si>
-    <t>44762009</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/02-EMZ-Emergentes y zoonóticos/44762009-Bacillus/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Clostridium botulinico</t>
-  </si>
-  <si>
-    <t>13080008</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/02-EMZ-Emergentes y zoonóticos/13080008-C.botulinico/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Mycobacterium leprae</t>
-  </si>
-  <si>
-    <t>58242002</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/07-MYCO-Mico Bacterias/58242002-M.leprae/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Clostridium tetanicum</t>
-  </si>
-  <si>
-    <t>30917009</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/02-EMZ-Emergentes y zoonóticos/30917009-C.tetanicum/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Corynebacterium Diphtheriae</t>
-  </si>
-  <si>
-    <t>5851001</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/02-EMZ-Emergentes y zoonóticos/5851001-C.Diphtheriae/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Mycobacterium tuberculosis</t>
-  </si>
-  <si>
-    <t>113861009</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/07-MYCO-Mico Bacterias/113861009-M.tuberculosis/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>VIH</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/03-Virus/06-Virus VIH/PENDIENTE-VIH/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>PCR Brucella spp</t>
-  </si>
-  <si>
-    <t>26250004_PCR</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/02-EMZ-Emergentes y zoonóticos/26250004-Brucella spp/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t>PCR Vibrio cholerae</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/03-ETA-Enfermedades Transmitidas por Alimentos/75953000-V. cholerae/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t>PCR Neisseria gonorrhoeae</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/05-ITS-Infecciones de Transmisión Sexual/68704007-N. gonorrhoeae/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t>PCR Mycobacterium leprae</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/07-MYCO-Mico Bacterias/58242002-M.leprae/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t>PCR Mycobacterium tuberculosis</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/07-MYCO-Mico Bacterias/113861009-M.tuberculosis/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Salmonella typhi y paratyphi
-</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/01-Bacterias/03-ETA-Enfermedades Transmitidas por Alimentos/_PENDIENTE_SalmonellaTP/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>PCR Cisticercosis</t>
-  </si>
-  <si>
-    <t>17966003</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/02-Parasitos/17966003-Cisticercosis/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t>PCR Hidatidosis</t>
-  </si>
-  <si>
-    <t>243672005</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/02-Parasitos/243672005-Hidatidosis/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t>PCR Leishmaniasis</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/02-Parasitos/7527002-Leishmaniasis/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t>PCR Trypanosoma cruzi (Chagas)</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/02-Parasitos/88274000-Trypanosoma_cruzi(Chagas)/Datos Vigilancia/PCR</t>
-  </si>
-  <si>
-    <t>Cisticercosis</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/02-Parasitos/17966003-Cisticercosis/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Hidatidosis</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/243672005-Hidatidosis/Datos Vigilancia</t>
-  </si>
-  <si>
-    <t>Leishmaniasis</t>
-  </si>
-  <si>
-    <t>/Documentos compartidos/Biomedico/02-Parasitos/7527002-Leishmaniasis/Datos Vigilancia</t>
+    <t>/Documentos compartidos/Biomedico/01-Bacterias/0-Otros/Diarrea</t>
+  </si>
+  <si>
+    <t>Sarampión-Rubéola</t>
+  </si>
+  <si>
+    <t>52584002-5210005</t>
+  </si>
+  <si>
+    <t>/Documentos compartidos/Biomedico/03-Virus/52584002-5210005_Sarampion-Rubeola/Datos Vigilancia</t>
   </si>
   <si>
     <t>Agente</t>
@@ -1216,22 +1110,25 @@
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="query (1)" backgroundRefresh="0" connectionId="1" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
-  <queryTableRefresh nextId="14">
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="query" backgroundRefresh="0" connectionId="1" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
+  <queryTableRefresh nextId="17">
     <queryTableFields count="3">
       <queryTableField id="1" name="Title" tableColumnId="1"/>
       <queryTableField id="2" name="SNOMED_CT" tableColumnId="2"/>
       <queryTableField id="6" name="RutaCarpeta" tableColumnId="7"/>
     </queryTableFields>
-    <queryTableDeletedFields count="10">
+    <queryTableDeletedFields count="13">
       <deletedField name="Departamento"/>
       <deletedField name="Seccion"/>
       <deletedField name="Laboratorio"/>
       <deletedField name="Sufijo"/>
+      <deletedField name="Periodicidad"/>
+      <deletedField name="EnvioCorreo"/>
+      <deletedField name="CorreoCC"/>
+      <deletedField name="TiposMuestra"/>
+      <deletedField name="MenuApp"/>
+      <deletedField name="DUDAS"/>
       <deletedField name="Vínculo"/>
-      <deletedField name="Periodicidad"/>
-      <deletedField name="Susceptibilidad"/>
-      <deletedField name="PCR"/>
       <deletedField name="Tipo de elemento"/>
       <deletedField name="Ruta de acceso"/>
     </queryTableDeletedFields>
@@ -1240,8 +1137,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla_query__1" displayName="Tabla_query__1" ref="A1:C74" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:C74"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla_query" displayName="Tabla_query" ref="A1:C58" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:C58"/>
   <tableColumns count="3">
     <tableColumn id="1" uniqueName="Title" name="Agente" queryTableFieldId="1" dataDxfId="2"/>
     <tableColumn id="2" uniqueName="field_1" name="SNOMED_CT" queryTableFieldId="2" dataDxfId="1"/>
@@ -1514,17 +1411,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="80.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>208</v>
+        <v>173</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1835,505 +1732,329 @@
         <v>83</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="B59" s="1" t="s">
         <v>172</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A74" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>207</v>
       </c>
     </row>
   </sheetData>

</xml_diff>